<commit_message>
tesntando nova função 00, encontrando as 100 redes
</commit_message>
<xml_diff>
--- a/fuction_ensemble/redes-ensemble-s/Teste05/content/results/metrics_22_8.xlsx
+++ b/fuction_ensemble/redes-ensemble-s/Teste05/content/results/metrics_22_8.xlsx
@@ -513,496 +513,496 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_15</t>
+          <t>model_22_8_3</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9954647642017688</v>
+        <v>0.9939432125889789</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8150438163676118</v>
+        <v>0.7572488114304166</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9940335706045256</v>
+        <v>0.9298736709298656</v>
       </c>
       <c r="E2" t="n">
-        <v>0.993577692761605</v>
+        <v>0.9905216355529797</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9940363129644438</v>
+        <v>0.9762402121922417</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03032714266561281</v>
+        <v>0.04050176530643978</v>
       </c>
       <c r="H2" t="n">
-        <v>1.236802851594697</v>
+        <v>1.623278315731249</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1353755607573606</v>
+        <v>0.1894930338644287</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01669115442382092</v>
+        <v>0.01138819312756301</v>
       </c>
       <c r="K2" t="n">
-        <v>0.07603335759059074</v>
+        <v>0.1004406137763513</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1556036340070171</v>
+        <v>0.2201325470192456</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1741468996726982</v>
+        <v>0.2012505038663004</v>
       </c>
       <c r="N2" t="n">
-        <v>1.001674548602424</v>
+        <v>1.001264025198822</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1815606937255442</v>
+        <v>0.2098181544618634</v>
       </c>
       <c r="P2" t="n">
-        <v>184.991424339818</v>
+        <v>284.4128194360125</v>
       </c>
       <c r="Q2" t="n">
-        <v>293.4713727530878</v>
+        <v>453.8365590926923</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_16</t>
+          <t>model_22_8_2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9953359408931085</v>
+        <v>0.9927334329859473</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8150406037342838</v>
+        <v>0.7564326753633799</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9936567498129519</v>
+        <v>0.9631137434527076</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9931187465431406</v>
+        <v>0.9978218405048332</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9936542292685723</v>
+        <v>0.9879013806330623</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03118858472380053</v>
+        <v>0.04859156708243489</v>
       </c>
       <c r="H3" t="n">
-        <v>1.236824334488554</v>
+        <v>1.628735821369485</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1439254525909941</v>
+        <v>0.09967281552778275</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01788392548261148</v>
+        <v>0.002617044441817375</v>
       </c>
       <c r="K3" t="n">
-        <v>0.08090469072804825</v>
+        <v>0.05114493298062502</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1512800476403452</v>
+        <v>0.2674669735909033</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1766029012326823</v>
+        <v>0.2204349497752906</v>
       </c>
       <c r="N3" t="n">
-        <v>1.001722114131775</v>
+        <v>1.001516500942063</v>
       </c>
       <c r="O3" t="n">
-        <v>0.184121252356561</v>
+        <v>0.2298193219504771</v>
       </c>
       <c r="P3" t="n">
-        <v>184.9354062507043</v>
+        <v>284.0486105599076</v>
       </c>
       <c r="Q3" t="n">
-        <v>293.4153546639741</v>
+        <v>453.4723502165875</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_14</t>
+          <t>model_22_8_4</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9955857777779382</v>
+        <v>0.993333394032145</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8150328417498344</v>
+        <v>0.7560973674364752</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9944200054293661</v>
+        <v>0.9092068273917778</v>
       </c>
       <c r="E4" t="n">
-        <v>0.994047586968093</v>
+        <v>0.9832784290453955</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9944280672325335</v>
+        <v>0.9686056245742425</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02951792432455153</v>
+        <v>0.04457962480394429</v>
       </c>
       <c r="H4" t="n">
-        <v>1.236876238914308</v>
+        <v>1.630978027020647</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1266075308953739</v>
+        <v>0.2453382910504574</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01546993026368376</v>
+        <v>0.02009085855388782</v>
       </c>
       <c r="K4" t="n">
-        <v>0.07103873057952881</v>
+        <v>0.1327145832446634</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1602108999001306</v>
+        <v>0.193631300375281</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1718078121755572</v>
+        <v>0.2111388756338924</v>
       </c>
       <c r="N4" t="n">
-        <v>1.001629866666607</v>
+        <v>1.001391291680248</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1791220264310713</v>
+        <v>0.2201274946873533</v>
       </c>
       <c r="P4" t="n">
-        <v>185.045515191862</v>
+        <v>284.2209567346031</v>
       </c>
       <c r="Q4" t="n">
-        <v>293.5254636051318</v>
+        <v>453.6446963912829</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_17</t>
+          <t>model_22_8_5</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9952014491313776</v>
+        <v>0.9926901266672501</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8150255672831792</v>
+        <v>0.75508755418947</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9932904053764188</v>
+        <v>0.8977194973654157</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9926721971557063</v>
+        <v>0.9785109942097446</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9932827315333106</v>
+        <v>0.9642567019821415</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03208793175377241</v>
+        <v>0.0488811566349707</v>
       </c>
       <c r="H5" t="n">
-        <v>1.236924883306327</v>
+        <v>1.637730652853133</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1522376407086705</v>
+        <v>0.2763789721549864</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01904447799230273</v>
+        <v>0.02581890044707879</v>
       </c>
       <c r="K5" t="n">
-        <v>0.08564105935048663</v>
+        <v>0.1510989416383789</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1472191293110307</v>
+        <v>0.1803723867732788</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1791310463146252</v>
+        <v>0.2210908334485414</v>
       </c>
       <c r="N5" t="n">
-        <v>1.001771772628414</v>
+        <v>1.001525538782487</v>
       </c>
       <c r="O5" t="n">
-        <v>0.186757025808624</v>
+        <v>0.2305031279495647</v>
       </c>
       <c r="P5" t="n">
-        <v>184.8785505547249</v>
+        <v>284.0367266033077</v>
       </c>
       <c r="Q5" t="n">
-        <v>293.3584989679947</v>
+        <v>453.4604662599876</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_13</t>
+          <t>model_22_8_6</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9956964072045152</v>
+        <v>0.9922811864861678</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8150049127512843</v>
+        <v>0.754468419187429</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9948148156161255</v>
+        <v>0.8916736843372548</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9945270568056978</v>
+        <v>0.9758182626797813</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9948282501241449</v>
+        <v>0.9619417575170508</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02877814483962915</v>
+        <v>0.05161574150886383</v>
       </c>
       <c r="H6" t="n">
-        <v>1.237063000256214</v>
+        <v>1.641870811462636</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1176494678927652</v>
+        <v>0.2927157670232524</v>
       </c>
       <c r="J6" t="n">
-        <v>0.01422381966760716</v>
+        <v>0.02905419983605098</v>
       </c>
       <c r="K6" t="n">
-        <v>0.06593664378018617</v>
+        <v>0.1608849904370112</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1651128148767088</v>
+        <v>0.173738895760265</v>
       </c>
       <c r="M6" t="n">
-        <v>0.169641223880368</v>
+        <v>0.227190980254199</v>
       </c>
       <c r="N6" t="n">
-        <v>1.001589018878333</v>
+        <v>1.001610882820278</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1768632019866999</v>
+        <v>0.2368629706337837</v>
       </c>
       <c r="P6" t="n">
-        <v>185.0962780793103</v>
+        <v>283.9278571700343</v>
       </c>
       <c r="Q6" t="n">
-        <v>293.5762264925801</v>
+        <v>453.3515968267142</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_18</t>
+          <t>model_22_8_7</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.995063176463976</v>
+        <v>0.9920546722055111</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8150008183569208</v>
+        <v>0.7541297132522337</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9929353036047825</v>
+        <v>0.8885743131838577</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9922389382631323</v>
+        <v>0.9743924818389565</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9929225924764703</v>
+        <v>0.9607485643434425</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03301256171737436</v>
+        <v>0.05313044354661781</v>
       </c>
       <c r="H7" t="n">
-        <v>1.237090379490175</v>
+        <v>1.644135739610884</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1602947378893817</v>
+        <v>0.3010907846623724</v>
       </c>
       <c r="J7" t="n">
-        <v>0.02017048937933413</v>
+        <v>0.03076726622673997</v>
       </c>
       <c r="K7" t="n">
-        <v>0.09023261177901262</v>
+        <v>0.1659290192675988</v>
       </c>
       <c r="L7" t="n">
-        <v>0.143401175309862</v>
+        <v>0.1704273331756388</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1816935929453055</v>
+        <v>0.2305004198404372</v>
       </c>
       <c r="N7" t="n">
-        <v>1.001822827151763</v>
+        <v>1.001658155365806</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1894286653545751</v>
+        <v>0.2403132999146924</v>
       </c>
       <c r="P7" t="n">
-        <v>184.8217342636906</v>
+        <v>283.8700103804541</v>
       </c>
       <c r="Q7" t="n">
-        <v>293.3016826769605</v>
+        <v>453.293750037134</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_19</t>
+          <t>model_22_8_8</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9949227341997279</v>
+        <v>0.9919358960018451</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8149681469094548</v>
+        <v>0.7539530290652611</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9925920506158333</v>
+        <v>0.887005432570152</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9918196620657046</v>
+        <v>0.9736599498112549</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9925744216869219</v>
+        <v>0.9601430379230147</v>
       </c>
       <c r="G8" t="n">
-        <v>0.03395169978507903</v>
+        <v>0.05392470056744642</v>
       </c>
       <c r="H8" t="n">
-        <v>1.237308853609818</v>
+        <v>1.645317227582726</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1680829915970146</v>
+        <v>0.305330161672466</v>
       </c>
       <c r="J8" t="n">
-        <v>0.02126016066065489</v>
+        <v>0.03164739868526909</v>
       </c>
       <c r="K8" t="n">
-        <v>0.09467157612883473</v>
+        <v>0.1684887830928339</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1398179517530709</v>
+        <v>0.1687741800497301</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1842598702514441</v>
+        <v>0.2322169256696127</v>
       </c>
       <c r="N8" t="n">
-        <v>1.001874682757024</v>
+        <v>1.001682943443093</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1921041943985625</v>
+        <v>0.2421028809506729</v>
       </c>
       <c r="P8" t="n">
-        <v>184.7656327178471</v>
+        <v>283.8403332789636</v>
       </c>
       <c r="Q8" t="n">
-        <v>293.245581131117</v>
+        <v>453.2640729356434</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_12</t>
+          <t>model_22_8_9</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9957936757501638</v>
+        <v>0.9918750754288874</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8149568650039736</v>
+        <v>0.7538628573618803</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9952164814716218</v>
+        <v>0.8862155548786046</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9950139652240828</v>
+        <v>0.9732884090697983</v>
       </c>
       <c r="F9" t="n">
-        <v>0.995235291556089</v>
+        <v>0.9598377875395144</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02812770962699751</v>
+        <v>0.0543314080188673</v>
       </c>
       <c r="H9" t="n">
-        <v>1.23738429576372</v>
+        <v>1.645920206178436</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1085358528944654</v>
+        <v>0.3074645428975755</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01295837668896273</v>
+        <v>0.03209380246538496</v>
       </c>
       <c r="K9" t="n">
-        <v>0.06074711479171407</v>
+        <v>0.1697791791234005</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1703296483675851</v>
+        <v>0.1679521763088017</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1677131766647973</v>
+        <v>0.2330909865671929</v>
       </c>
       <c r="N9" t="n">
-        <v>1.001553104338401</v>
+        <v>1.001695636432232</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1748530738095544</v>
+        <v>0.2430141524302186</v>
       </c>
       <c r="P9" t="n">
-        <v>185.1420001616099</v>
+        <v>283.8253056054138</v>
       </c>
       <c r="Q9" t="n">
-        <v>293.6219485748797</v>
+        <v>453.2490452620937</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_20</t>
+          <t>model_22_8_10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9947813952937796</v>
+        <v>0.9918443373921656</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8149291142408316</v>
+        <v>0.753817297977403</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9922609017132529</v>
+        <v>0.8858197502988144</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9914149519797832</v>
+        <v>0.9731012737325238</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9922385058966379</v>
+        <v>0.9596846942453773</v>
       </c>
       <c r="G10" t="n">
-        <v>0.03489683369996063</v>
+        <v>0.05453695341196196</v>
       </c>
       <c r="H10" t="n">
-        <v>1.237569865244631</v>
+        <v>1.646224861992217</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1755966091075181</v>
+        <v>0.3085340728677933</v>
       </c>
       <c r="J10" t="n">
-        <v>0.02231197557548901</v>
+        <v>0.03231864435385489</v>
       </c>
       <c r="K10" t="n">
-        <v>0.09895429674289735</v>
+        <v>0.1704263559649024</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1364508599450066</v>
+        <v>0.1675370420774842</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1868069423227109</v>
+        <v>0.2335314826997892</v>
       </c>
       <c r="N10" t="n">
-        <v>1.001926869429989</v>
+        <v>1.001702051326852</v>
       </c>
       <c r="O10" t="n">
-        <v>0.1947597006010691</v>
+        <v>0.2434734013951322</v>
       </c>
       <c r="P10" t="n">
-        <v>184.710718357638</v>
+        <v>283.8177535256498</v>
       </c>
       <c r="Q10" t="n">
-        <v>293.1906667709079</v>
+        <v>453.2414931823297</v>
       </c>
     </row>
     <row r="11">
@@ -1012,767 +1012,767 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9958741204024574</v>
+        <v>0.9918288813382942</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8148850548937621</v>
+        <v>0.7537943804449907</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9956231340852033</v>
+        <v>0.8856214665288288</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9955061763093729</v>
+        <v>0.9730075565313744</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9956473108172589</v>
+        <v>0.9596080011488015</v>
       </c>
       <c r="G11" t="n">
-        <v>0.02758977586669637</v>
+        <v>0.05464030811536905</v>
       </c>
       <c r="H11" t="n">
-        <v>1.23786449030136</v>
+        <v>1.646378111636984</v>
       </c>
       <c r="I11" t="n">
-        <v>0.09930909063045434</v>
+        <v>0.3090698686757141</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01167915242753593</v>
+        <v>0.03243124496042894</v>
       </c>
       <c r="K11" t="n">
-        <v>0.05549412152899513</v>
+        <v>0.1707505634769729</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1758824691224331</v>
+        <v>0.1673307899458543</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1661017033828864</v>
+        <v>0.2337526644027166</v>
       </c>
       <c r="N11" t="n">
-        <v>1.001523401697554</v>
+        <v>1.001705276938095</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1731729967738229</v>
+        <v>0.2437039992610625</v>
       </c>
       <c r="P11" t="n">
-        <v>185.1806200290024</v>
+        <v>283.8139668494561</v>
       </c>
       <c r="Q11" t="n">
-        <v>293.6605684422722</v>
+        <v>453.2377065061359</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_21</t>
+          <t>model_22_8_12</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9946403265629684</v>
+        <v>0.9918211404387594</v>
       </c>
       <c r="C12" t="n">
-        <v>0.8148850483107968</v>
+        <v>0.7537829149869028</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9919421762052135</v>
+        <v>0.8855223335298428</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9910250755780678</v>
+        <v>0.9729607336041103</v>
       </c>
       <c r="F12" t="n">
-        <v>0.991915157397413</v>
+        <v>0.9595696664461919</v>
       </c>
       <c r="G12" t="n">
-        <v>0.03584016095245719</v>
+        <v>0.05469207154620187</v>
       </c>
       <c r="H12" t="n">
-        <v>1.237864534321678</v>
+        <v>1.646454781208012</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1828283454641449</v>
+        <v>0.3093377425682025</v>
       </c>
       <c r="J12" t="n">
-        <v>0.02332523871997562</v>
+        <v>0.03248750240246567</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1030767920920602</v>
+        <v>0.1709126171573421</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1335396155304631</v>
+        <v>0.1672273249077045</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1893149781513792</v>
+        <v>0.2338633608460331</v>
       </c>
       <c r="N12" t="n">
-        <v>1.001978956345981</v>
+        <v>1.001706892430172</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1973745087073137</v>
+        <v>0.2438194082811441</v>
       </c>
       <c r="P12" t="n">
-        <v>184.657372400049</v>
+        <v>283.8120730487408</v>
       </c>
       <c r="Q12" t="n">
-        <v>293.1373208133189</v>
+        <v>453.2358127054206</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_22</t>
+          <t>model_22_8_13</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.9945004255145097</v>
+        <v>0.9918172554429897</v>
       </c>
       <c r="C13" t="n">
-        <v>0.8148371128739428</v>
+        <v>0.7537771960682762</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9916359160882922</v>
+        <v>0.8854726910467147</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9906501419871017</v>
+        <v>0.9729371148481343</v>
       </c>
       <c r="F13" t="n">
-        <v>0.9916044236459393</v>
+        <v>0.9595504405146251</v>
       </c>
       <c r="G13" t="n">
-        <v>0.03677567990768615</v>
+        <v>0.0547180505308022</v>
       </c>
       <c r="H13" t="n">
-        <v>1.238185078808643</v>
+        <v>1.646493023643201</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1897772477837278</v>
+        <v>0.3094718848348982</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02429966648140074</v>
+        <v>0.03251588018388473</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1070384571325643</v>
+        <v>0.1709938916359956</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1309570963447985</v>
+        <v>0.16717576887385</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1917698618336212</v>
+        <v>0.2339188973358121</v>
       </c>
       <c r="N13" t="n">
-        <v>1.00203061211772</v>
+        <v>1.001707703211898</v>
       </c>
       <c r="O13" t="n">
-        <v>0.1999339018702185</v>
+        <v>0.2438773090742694</v>
       </c>
       <c r="P13" t="n">
-        <v>184.6058370487064</v>
+        <v>283.8111232651341</v>
       </c>
       <c r="Q13" t="n">
-        <v>293.0857854619762</v>
+        <v>453.2348629218139</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_23</t>
+          <t>model_22_8_14</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9943624629472316</v>
+        <v>0.9918153058770472</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8147862668184568</v>
+        <v>0.7537742149881643</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9913421547374333</v>
+        <v>0.8854476739434327</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9902902387287572</v>
+        <v>0.9729255314055645</v>
       </c>
       <c r="F14" t="n">
-        <v>0.9913063436059956</v>
+        <v>0.9595408006135695</v>
       </c>
       <c r="G14" t="n">
-        <v>0.03769823623033369</v>
+        <v>0.05473108728723652</v>
       </c>
       <c r="H14" t="n">
-        <v>1.238525086615803</v>
+        <v>1.646512958139635</v>
       </c>
       <c r="I14" t="n">
-        <v>0.196442558804007</v>
+        <v>0.3095394852192651</v>
       </c>
       <c r="J14" t="n">
-        <v>0.02523503139617008</v>
+        <v>0.03252979761466127</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1108387951000885</v>
+        <v>0.1710346427397767</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1285307228558157</v>
+        <v>0.1671498784524054</v>
       </c>
       <c r="M14" t="n">
-        <v>0.1941603363983841</v>
+        <v>0.2339467616515273</v>
       </c>
       <c r="N14" t="n">
-        <v>1.002081552142561</v>
+        <v>1.001708110077834</v>
       </c>
       <c r="O14" t="n">
-        <v>0.202426143886168</v>
+        <v>0.2439063596315917</v>
       </c>
       <c r="P14" t="n">
-        <v>184.5562839399277</v>
+        <v>283.8106468152778</v>
       </c>
       <c r="Q14" t="n">
-        <v>293.0362323531976</v>
+        <v>453.2343864719577</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_10</t>
+          <t>model_22_8_15</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.995933734202717</v>
+        <v>0.9918143433041339</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8147852978594431</v>
+        <v>0.7537728033855208</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9960325909686383</v>
+        <v>0.8854354504381959</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9960005665631633</v>
+        <v>0.9729195311435153</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9960620476914462</v>
+        <v>0.959536044309954</v>
       </c>
       <c r="G15" t="n">
-        <v>0.02719113810986382</v>
+        <v>0.05473752401673981</v>
       </c>
       <c r="H15" t="n">
-        <v>1.238531566049189</v>
+        <v>1.646522397533013</v>
       </c>
       <c r="I15" t="n">
-        <v>0.09001870076293972</v>
+        <v>0.3095725151685367</v>
       </c>
       <c r="J15" t="n">
-        <v>0.01039426465039634</v>
+        <v>0.03253700689041917</v>
       </c>
       <c r="K15" t="n">
-        <v>0.05020648036454788</v>
+        <v>0.1710547492347637</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1818048376389743</v>
+        <v>0.1671325909667304</v>
       </c>
       <c r="M15" t="n">
-        <v>0.1648973562852474</v>
+        <v>0.2339605180724727</v>
       </c>
       <c r="N15" t="n">
-        <v>1.001501390448228</v>
+        <v>1.001708310962615</v>
       </c>
       <c r="O15" t="n">
-        <v>0.1719173781268953</v>
+        <v>0.2439207016918565</v>
       </c>
       <c r="P15" t="n">
-        <v>185.209728327101</v>
+        <v>283.8104116161853</v>
       </c>
       <c r="Q15" t="n">
-        <v>293.6896767403708</v>
+        <v>453.2341512728651</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_24</t>
+          <t>model_22_8_16</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.9942270516041014</v>
+        <v>0.9918138886215156</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8147333933507062</v>
+        <v>0.7537720635233585</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9910607705037882</v>
+        <v>0.8854297256329349</v>
       </c>
       <c r="E16" t="n">
-        <v>0.9899454036036281</v>
+        <v>0.9729165883633536</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9910208128837203</v>
+        <v>0.9595337908018923</v>
       </c>
       <c r="G16" t="n">
-        <v>0.03860373250535732</v>
+        <v>0.05474056448150186</v>
       </c>
       <c r="H16" t="n">
-        <v>1.238878651738112</v>
+        <v>1.646527344994699</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2028270386818513</v>
+        <v>0.3095879845468941</v>
       </c>
       <c r="J16" t="n">
-        <v>0.02613123522302505</v>
+        <v>0.03254054262160996</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1144791369524382</v>
+        <v>0.1710642755712233</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1262511938385172</v>
+        <v>0.1671291614356429</v>
       </c>
       <c r="M16" t="n">
-        <v>0.1964783257902951</v>
+        <v>0.2339670157981716</v>
       </c>
       <c r="N16" t="n">
-        <v>1.002131550176947</v>
+        <v>1.001708405852901</v>
       </c>
       <c r="O16" t="n">
-        <v>0.204842814885392</v>
+        <v>0.2439274760391905</v>
       </c>
       <c r="P16" t="n">
-        <v>184.5088126203125</v>
+        <v>283.8103005267498</v>
       </c>
       <c r="Q16" t="n">
-        <v>292.9887610335823</v>
+        <v>453.2340401834296</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_9</t>
+          <t>model_22_8_17</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.9959678978993152</v>
+        <v>0.9918135905136357</v>
       </c>
       <c r="C17" t="n">
-        <v>0.8146528438445364</v>
+        <v>0.7537717413323091</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9964421130147655</v>
+        <v>0.8854255589065285</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9964937873350177</v>
+        <v>0.9729155891702341</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9964767231307636</v>
+        <v>0.9595323222241599</v>
       </c>
       <c r="G17" t="n">
-        <v>0.02696268531340267</v>
+        <v>0.05474255793026737</v>
       </c>
       <c r="H17" t="n">
-        <v>1.239417286656765</v>
+        <v>1.646529499487729</v>
       </c>
       <c r="I17" t="n">
-        <v>0.08072683238366696</v>
+        <v>0.3095992437363952</v>
       </c>
       <c r="J17" t="n">
-        <v>0.009112416279947595</v>
+        <v>0.03254174314563283</v>
       </c>
       <c r="K17" t="n">
-        <v>0.04491962245707026</v>
+        <v>0.1710704837431993</v>
       </c>
       <c r="L17" t="n">
-        <v>0.1881022777382841</v>
+        <v>0.1671284956611654</v>
       </c>
       <c r="M17" t="n">
-        <v>0.1642031830184868</v>
+        <v>0.2339712758657938</v>
       </c>
       <c r="N17" t="n">
-        <v>1.001488776160253</v>
+        <v>1.001708468066719</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1711936524670319</v>
+        <v>0.2439319174667109</v>
       </c>
       <c r="P17" t="n">
-        <v>185.2266027885706</v>
+        <v>283.8102276954778</v>
       </c>
       <c r="Q17" t="n">
-        <v>293.7065512018404</v>
+        <v>453.2339673521577</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_8</t>
+          <t>model_22_8_24</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.9959712543907042</v>
+        <v>0.9918133986212622</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8144822713753023</v>
+        <v>0.7537715931996664</v>
       </c>
       <c r="D18" t="n">
-        <v>0.9968484927226066</v>
+        <v>0.8854234899378759</v>
       </c>
       <c r="E18" t="n">
-        <v>0.9969816154632924</v>
+        <v>0.9729135671955008</v>
       </c>
       <c r="F18" t="n">
-        <v>0.9968880526774949</v>
+        <v>0.9595313684948584</v>
       </c>
       <c r="G18" t="n">
-        <v>0.02694024044002898</v>
+        <v>0.05474384111545316</v>
       </c>
       <c r="H18" t="n">
-        <v>1.240557905543947</v>
+        <v>1.646530490051394</v>
       </c>
       <c r="I18" t="n">
-        <v>0.07150626222639042</v>
+        <v>0.3096048344346701</v>
       </c>
       <c r="J18" t="n">
-        <v>0.007844583035745359</v>
+        <v>0.03254417253510085</v>
       </c>
       <c r="K18" t="n">
-        <v>0.03967542263106789</v>
+        <v>0.1710745154777077</v>
       </c>
       <c r="L18" t="n">
-        <v>0.194814965416297</v>
+        <v>0.1671257595514889</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1641348239711152</v>
+        <v>0.2339740180350228</v>
       </c>
       <c r="N18" t="n">
-        <v>1.001487536840355</v>
+        <v>1.001708508113824</v>
       </c>
       <c r="O18" t="n">
-        <v>0.171122383233491</v>
+        <v>0.2439347763757611</v>
       </c>
       <c r="P18" t="n">
-        <v>185.2282683660402</v>
+        <v>283.8101808153102</v>
       </c>
       <c r="Q18" t="n">
-        <v>293.70821677931</v>
+        <v>453.23392047199</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_7</t>
+          <t>model_22_8_23</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.9959377211484028</v>
+        <v>0.9918133986212622</v>
       </c>
       <c r="C19" t="n">
-        <v>0.8142673220992923</v>
+        <v>0.7537715931996664</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9972480093318357</v>
+        <v>0.8854234899378759</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9974592808236497</v>
+        <v>0.9729135671955008</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9972922395598806</v>
+        <v>0.9595313684948584</v>
       </c>
       <c r="G19" t="n">
-        <v>0.02716447738570413</v>
+        <v>0.05474384111545316</v>
       </c>
       <c r="H19" t="n">
-        <v>1.241995272342377</v>
+        <v>1.646530490051394</v>
       </c>
       <c r="I19" t="n">
-        <v>0.06244141264528563</v>
+        <v>0.3096048344346701</v>
       </c>
       <c r="J19" t="n">
-        <v>0.006603162157440635</v>
+        <v>0.03254417253510085</v>
       </c>
       <c r="K19" t="n">
-        <v>0.03452228740136313</v>
+        <v>0.1710745154777077</v>
       </c>
       <c r="L19" t="n">
-        <v>0.2019579324408196</v>
+        <v>0.1671257595514889</v>
       </c>
       <c r="M19" t="n">
-        <v>0.1648164960970355</v>
+        <v>0.2339740180350228</v>
       </c>
       <c r="N19" t="n">
-        <v>1.001499918345205</v>
+        <v>1.001708508113824</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1718330755530676</v>
+        <v>0.2439347763757611</v>
       </c>
       <c r="P19" t="n">
-        <v>185.2116902753601</v>
+        <v>283.8101808153102</v>
       </c>
       <c r="Q19" t="n">
-        <v>293.6916386886299</v>
+        <v>453.23392047199</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_6</t>
+          <t>model_22_8_21</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.9958602311546736</v>
+        <v>0.9918134071205317</v>
       </c>
       <c r="C20" t="n">
-        <v>0.8140009700120808</v>
+        <v>0.7537715785408219</v>
       </c>
       <c r="D20" t="n">
-        <v>0.9976361975531788</v>
+        <v>0.8854235508360488</v>
       </c>
       <c r="E20" t="n">
-        <v>0.9979210046898215</v>
+        <v>0.9729137258805166</v>
       </c>
       <c r="F20" t="n">
-        <v>0.9976847212977794</v>
+        <v>0.9595314143358196</v>
       </c>
       <c r="G20" t="n">
-        <v>0.02768265333058062</v>
+        <v>0.05474378428079893</v>
       </c>
       <c r="H20" t="n">
-        <v>1.243776369975998</v>
+        <v>1.646530588075154</v>
       </c>
       <c r="I20" t="n">
-        <v>0.053633599016652</v>
+        <v>0.3096046698776526</v>
       </c>
       <c r="J20" t="n">
-        <v>0.005403172174811986</v>
+        <v>0.03254398187608829</v>
       </c>
       <c r="K20" t="n">
-        <v>0.02951838559573199</v>
+        <v>0.171074321692548</v>
       </c>
       <c r="L20" t="n">
-        <v>0.20957165624678</v>
+        <v>0.1671252272283743</v>
       </c>
       <c r="M20" t="n">
-        <v>0.1663810485920215</v>
+        <v>0.2339738965799367</v>
       </c>
       <c r="N20" t="n">
-        <v>1.001528530035197</v>
+        <v>1.001708506340063</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1734642342868352</v>
+        <v>0.2439346497500806</v>
       </c>
       <c r="P20" t="n">
-        <v>185.173898591016</v>
+        <v>283.8101828916966</v>
       </c>
       <c r="Q20" t="n">
-        <v>293.6538470042859</v>
+        <v>453.2339225483764</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_5</t>
+          <t>model_22_8_22</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.9957307325377045</v>
+        <v>0.991813408405039</v>
       </c>
       <c r="C21" t="n">
-        <v>0.8136751797436881</v>
+        <v>0.7537715722134541</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9980079005076193</v>
+        <v>0.8854235710583264</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9983601053618951</v>
+        <v>0.9729137250819671</v>
       </c>
       <c r="F21" t="n">
-        <v>0.9980602281270625</v>
+        <v>0.9595314215406848</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0285486111785392</v>
+        <v>0.05474377569129283</v>
       </c>
       <c r="H21" t="n">
-        <v>1.245954931000866</v>
+        <v>1.646530630386291</v>
       </c>
       <c r="I21" t="n">
-        <v>0.04519982857251885</v>
+        <v>0.309604615233687</v>
       </c>
       <c r="J21" t="n">
-        <v>0.004261978386796337</v>
+        <v>0.03254398283554045</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0247309034796576</v>
+        <v>0.1710742912351594</v>
       </c>
       <c r="L21" t="n">
-        <v>0.2176834463375275</v>
+        <v>0.1671248045855772</v>
       </c>
       <c r="M21" t="n">
-        <v>0.1689633427064557</v>
+        <v>0.2339738782242429</v>
       </c>
       <c r="N21" t="n">
-        <v>1.001576344909155</v>
+        <v>1.001708506071992</v>
       </c>
       <c r="O21" t="n">
-        <v>0.1761564620078066</v>
+        <v>0.2439346306129468</v>
       </c>
       <c r="P21" t="n">
-        <v>185.1122939785968</v>
+        <v>283.8101832055041</v>
       </c>
       <c r="Q21" t="n">
-        <v>293.5922423918666</v>
+        <v>453.233922862184</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_4</t>
+          <t>model_22_8_18</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.9955400909410547</v>
+        <v>0.9918134676598317</v>
       </c>
       <c r="C22" t="n">
-        <v>0.8132807855625377</v>
+        <v>0.7537715380963389</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9983571736915153</v>
+        <v>0.8854240221127375</v>
       </c>
       <c r="E22" t="n">
-        <v>0.9987688927757092</v>
+        <v>0.9729147718653396</v>
       </c>
       <c r="F22" t="n">
-        <v>0.9984126866561475</v>
+        <v>0.9595317132461093</v>
       </c>
       <c r="G22" t="n">
-        <v>0.02982343241316074</v>
+        <v>0.05474337945422053</v>
       </c>
       <c r="H22" t="n">
-        <v>1.248592246706238</v>
+        <v>1.646530858527598</v>
       </c>
       <c r="I22" t="n">
-        <v>0.03727497938830016</v>
+        <v>0.3096033964094602</v>
       </c>
       <c r="J22" t="n">
-        <v>0.003199566764740174</v>
+        <v>0.03254272513213859</v>
       </c>
       <c r="K22" t="n">
-        <v>0.02023727307652017</v>
+        <v>0.1710730580982259</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2263174177323728</v>
+        <v>0.1671271487632728</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1726946218420271</v>
+        <v>0.2339730314677752</v>
       </c>
       <c r="N22" t="n">
-        <v>1.001646735652534</v>
+        <v>1.001708493705774</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1800465894209919</v>
+        <v>0.2439337478083033</v>
       </c>
       <c r="P22" t="n">
-        <v>185.0249217437423</v>
+        <v>283.8101976816158</v>
       </c>
       <c r="Q22" t="n">
-        <v>293.5048701570121</v>
+        <v>453.2339373382957</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_3</t>
+          <t>model_22_8_20</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.9952777838843828</v>
+        <v>0.9918134168901492</v>
       </c>
       <c r="C23" t="n">
-        <v>0.8128074623568201</v>
+        <v>0.7537714835357018</v>
       </c>
       <c r="D23" t="n">
-        <v>0.9986771068476418</v>
+        <v>0.8854235409044644</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9991382426400621</v>
+        <v>0.9729140880604518</v>
       </c>
       <c r="F23" t="n">
-        <v>0.9987350179561364</v>
+        <v>0.9595314616411864</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03157748090893765</v>
+        <v>0.05474371895132139</v>
       </c>
       <c r="H23" t="n">
-        <v>1.251757361162324</v>
+        <v>1.646531223374829</v>
       </c>
       <c r="I23" t="n">
-        <v>0.03001584204757409</v>
+        <v>0.3096046967144498</v>
       </c>
       <c r="J23" t="n">
-        <v>0.002239650741807507</v>
+        <v>0.03254354671925594</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0161277463946908</v>
+        <v>0.1710741217168529</v>
       </c>
       <c r="L23" t="n">
-        <v>0.2355222781183088</v>
+        <v>0.1671273274148891</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1777005371655855</v>
+        <v>0.2339737569714206</v>
       </c>
       <c r="N23" t="n">
-        <v>1.001743587488843</v>
+        <v>1.001708504301186</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1852656169235475</v>
+        <v>0.2439345041981409</v>
       </c>
       <c r="P23" t="n">
-        <v>184.9106220837887</v>
+        <v>283.8101852784339</v>
       </c>
       <c r="Q23" t="n">
-        <v>293.3905704970585</v>
+        <v>453.2339249351137</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>model_22_8_2</t>
+          <t>model_22_8_19</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.9949318868801704</v>
+        <v>0.991813444945836</v>
       </c>
       <c r="C24" t="n">
-        <v>0.8122434356810047</v>
+        <v>0.7537714352121908</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9989597748064848</v>
+        <v>0.8854237609861014</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9994577753961745</v>
+        <v>0.9729145690116288</v>
       </c>
       <c r="F24" t="n">
-        <v>0.9990191120582288</v>
+        <v>0.9595316038839776</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0338904957688152</v>
+        <v>0.05474353134281439</v>
       </c>
       <c r="H24" t="n">
-        <v>1.255529010140606</v>
+        <v>1.64653154651437</v>
       </c>
       <c r="I24" t="n">
-        <v>0.02360223503069832</v>
+        <v>0.3096041020171706</v>
       </c>
       <c r="J24" t="n">
-        <v>0.001409206109097432</v>
+        <v>0.03254296885955046</v>
       </c>
       <c r="K24" t="n">
-        <v>0.01250572056989788</v>
+        <v>0.1710735204087365</v>
       </c>
       <c r="L24" t="n">
-        <v>0.2455069852242737</v>
+        <v>0.1671268592310753</v>
       </c>
       <c r="M24" t="n">
-        <v>0.1840937146369077</v>
+        <v>0.2339733560532361</v>
       </c>
       <c r="N24" t="n">
-        <v>1.001871303305783</v>
+        <v>1.001708498446086</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1919309651955257</v>
+        <v>0.2439340862120393</v>
       </c>
       <c r="P24" t="n">
-        <v>184.7692413294122</v>
+        <v>283.8101921325107</v>
       </c>
       <c r="Q24" t="n">
-        <v>293.249189742682</v>
+        <v>453.2339317891906</v>
       </c>
     </row>
     <row r="25">
@@ -1782,52 +1782,52 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.9944888544341915</v>
+        <v>0.983637824795325</v>
       </c>
       <c r="C25" t="n">
-        <v>0.8115754248334115</v>
+        <v>0.7423242310555536</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9991961413538886</v>
+        <v>0.999980934001001</v>
       </c>
       <c r="E25" t="n">
-        <v>0.9997154406062465</v>
+        <v>0.9998654963288276</v>
       </c>
       <c r="F25" t="n">
-        <v>0.999255700051655</v>
+        <v>0.9999747920703331</v>
       </c>
       <c r="G25" t="n">
-        <v>0.03685305577505293</v>
+        <v>0.1094139409345506</v>
       </c>
       <c r="H25" t="n">
-        <v>1.259996001754369</v>
+        <v>1.723079053419331</v>
       </c>
       <c r="I25" t="n">
-        <v>0.01823918591402935</v>
+        <v>5.151950832010947e-05</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0007395511624689753</v>
+        <v>0.0001616052845656001</v>
       </c>
       <c r="K25" t="n">
-        <v>0.009489368538249162</v>
+        <v>0.0001065623964428548</v>
       </c>
       <c r="L25" t="n">
-        <v>0.2561454369451499</v>
+        <v>0.250237225526512</v>
       </c>
       <c r="M25" t="n">
-        <v>0.1919714972985649</v>
+        <v>0.3307777818030567</v>
       </c>
       <c r="N25" t="n">
-        <v>1.002034884516606</v>
+        <v>1.003414714825323</v>
       </c>
       <c r="O25" t="n">
-        <v>0.2001441213743479</v>
+        <v>0.3448596767788165</v>
       </c>
       <c r="P25" t="n">
-        <v>184.6016334781774</v>
+        <v>282.4252339325338</v>
       </c>
       <c r="Q25" t="n">
-        <v>293.0815818914472</v>
+        <v>451.8489735892136</v>
       </c>
     </row>
     <row r="26">
@@ -1837,52 +1837,52 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.9939333247729243</v>
+        <v>0.9835941292261904</v>
       </c>
       <c r="C26" t="n">
-        <v>0.810788453994349</v>
+        <v>0.7422542209503188</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9993759030610323</v>
+        <v>0.9999823678693488</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9998974421876029</v>
+        <v>0.9998650860312432</v>
       </c>
       <c r="F26" t="n">
-        <v>0.9994342074986703</v>
+        <v>0.9999751918568315</v>
       </c>
       <c r="G26" t="n">
-        <v>0.04056788517792624</v>
+        <v>0.1097061334065536</v>
       </c>
       <c r="H26" t="n">
-        <v>1.265258479378847</v>
+        <v>1.723547211315403</v>
       </c>
       <c r="I26" t="n">
-        <v>0.01416047479649948</v>
+        <v>4.764495696395432e-05</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0002665410140853973</v>
+        <v>0.0001620982544399903</v>
       </c>
       <c r="K26" t="n">
-        <v>0.007213507905292437</v>
+        <v>0.0001048723644610394</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2674765358541109</v>
+        <v>0.2489012165364721</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2014147094378319</v>
+        <v>0.3312191621971073</v>
       </c>
       <c r="N26" t="n">
-        <v>1.002240003160766</v>
+        <v>1.003423833900621</v>
       </c>
       <c r="O26" t="n">
-        <v>0.2099893506045274</v>
+        <v>0.3453198476500252</v>
       </c>
       <c r="P26" t="n">
-        <v>184.4095570617083</v>
+        <v>282.4199000050774</v>
       </c>
       <c r="Q26" t="n">
-        <v>292.8895054749781</v>
+        <v>451.8436396617573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>